<commit_message>
apply xlookup in excel
</commit_message>
<xml_diff>
--- a/finance_customer.csv.xlsx
+++ b/finance_customer.csv.xlsx
@@ -8,19 +8,54 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pandas\Finance data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BA9599C-D9A1-4FDD-8E4C-58C8540AB72E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3CF0C8-C512-4166-A190-319522D936ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9802DE5F-B1D8-4319-BDEA-30F1B831059A}"/>
   </bookViews>
   <sheets>
     <sheet name="finance_customer" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3138" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3158" uniqueCount="720">
   <si>
     <t>customer_id</t>
   </si>
@@ -2171,13 +2206,22 @@
   </si>
   <si>
     <t>Tol_cur_bal</t>
+  </si>
+  <si>
+    <t>customer _id</t>
+  </si>
+  <si>
+    <t>Emp_title</t>
+  </si>
+  <si>
+    <t>tot_cur_bal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2308,6 +2352,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2693,7 +2743,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2711,6 +2761,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3086,7 +3137,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{383771C4-FF3C-4B99-8491-974F447FF532}">
-  <dimension ref="A1:Q395"/>
+  <dimension ref="A1:W395"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -3094,19 +3145,27 @@
     <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.88671875" customWidth="1"/>
+    <col min="18" max="18" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3141,7 +3200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
@@ -3176,7 +3235,7 @@
         <v>34322</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -3211,7 +3270,7 @@
         <v>150674</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -3246,7 +3305,7 @@
         <v>281735</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
@@ -3281,7 +3340,7 @@
         <v>379132</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -3324,11 +3383,12 @@
       <c r="P6" s="7" t="s">
         <v>715</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7" t="s">
         <v>716</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
@@ -3367,19 +3427,20 @@
         <v>38335069.949000001</v>
       </c>
       <c r="O7" s="8">
-        <f t="shared" ref="O7:Q7" si="0">SUM(F1:F394)</f>
+        <f t="shared" ref="O7" si="0">SUM(F1:F394)</f>
         <v>3110000</v>
       </c>
       <c r="P7" s="8">
         <f>SUM(J1:J394)</f>
         <v>3202883</v>
       </c>
-      <c r="Q7" s="8">
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8">
         <f>SUM(K1:K394)</f>
         <v>32568773</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>36</v>
       </c>
@@ -3414,7 +3475,7 @@
         <v>408091</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>38</v>
       </c>
@@ -3449,7 +3510,7 @@
         <v>24448</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>40</v>
       </c>
@@ -3484,7 +3545,7 @@
         <v>30491</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>42</v>
       </c>
@@ -3519,7 +3580,7 @@
         <v>5927</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>44</v>
       </c>
@@ -3554,7 +3615,7 @@
         <v>96087</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>46</v>
       </c>
@@ -3589,7 +3650,7 @@
         <v>40264</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>48</v>
       </c>
@@ -3624,7 +3685,7 @@
         <v>5714</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>50</v>
       </c>
@@ -3659,7 +3720,7 @@
         <v>16656</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>52</v>
       </c>
@@ -3694,7 +3755,7 @@
         <v>37575</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>54</v>
       </c>
@@ -3728,8 +3789,41 @@
       <c r="K17" s="2">
         <v>142362</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M17" s="9" t="s">
+        <v>717</v>
+      </c>
+      <c r="N17" s="9" t="s">
+        <v>718</v>
+      </c>
+      <c r="O17" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="P17" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q17" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="R17" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="S17" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="T17" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="U17" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="V17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="W17" s="9" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>55</v>
       </c>
@@ -3763,8 +3857,42 @@
       <c r="K18" s="2">
         <v>76641</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M18" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="N18" s="2" t="str" cm="1">
+        <f t="array" ref="N18:W18">_xlfn.XLOOKUP(M18,A2:A394,B2:K394,"not found",0)</f>
+        <v>Mechanical</v>
+      </c>
+      <c r="O18" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P18" s="2" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>49000</v>
+      </c>
+      <c r="R18" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S18" s="2" t="str">
+        <v>Source Verified</v>
+      </c>
+      <c r="T18" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U18" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V18" s="2">
+        <v>2192</v>
+      </c>
+      <c r="W18" s="2">
+        <v>19731</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>57</v>
       </c>
@@ -3798,8 +3926,42 @@
       <c r="K19" s="2">
         <v>69267</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M19" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="N19" s="2" t="str" cm="1">
+        <f t="array" ref="N19:W19">_xlfn.XLOOKUP(M19,A3:A395,B3:K395,"not found",0)</f>
+        <v>Corrections Officer</v>
+      </c>
+      <c r="O19" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P19" s="2" t="str">
+        <v>Mortgage</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>74000</v>
+      </c>
+      <c r="R19" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S19" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="T19" s="2" t="str">
+        <v>107xx</v>
+      </c>
+      <c r="U19" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V19" s="2">
+        <v>47824</v>
+      </c>
+      <c r="W19" s="2">
+        <v>382595</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>59</v>
       </c>
@@ -3833,8 +3995,42 @@
       <c r="K20" s="2">
         <v>7013</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M20" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="N20" s="2" t="str" cm="1">
+        <f t="array" ref="N20:W20">_xlfn.XLOOKUP(M20,A4:A396,B4:K396,"not found",0)</f>
+        <v xml:space="preserve">Claims Adjuster </v>
+      </c>
+      <c r="O20" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P20" s="2" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>38000</v>
+      </c>
+      <c r="R20" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S20" s="2" t="str">
+        <v>Not Verified</v>
+      </c>
+      <c r="T20" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U20" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V20" s="2">
+        <v>1381</v>
+      </c>
+      <c r="W20" s="2">
+        <v>19340</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>61</v>
       </c>
@@ -3868,8 +4064,42 @@
       <c r="K21" s="2">
         <v>28818</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M21" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="N21" s="2" t="str" cm="1">
+        <f t="array" ref="N21:W21">_xlfn.XLOOKUP(M21,A5:A397,B5:K397,"not found",0)</f>
+        <v>Csr</v>
+      </c>
+      <c r="O21" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P21" s="2" t="str">
+        <v>Mortgage</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>65000</v>
+      </c>
+      <c r="R21" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S21" s="2" t="str">
+        <v>Not Verified</v>
+      </c>
+      <c r="T21" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U21" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V21" s="2">
+        <v>20384</v>
+      </c>
+      <c r="W21" s="2">
+        <v>448449</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>62</v>
       </c>
@@ -3903,8 +4133,42 @@
       <c r="K22" s="2">
         <v>36059</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M22" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="N22" s="2" t="str" cm="1">
+        <f t="array" ref="N22:W22">_xlfn.XLOOKUP(M22,A6:A398,B6:K398,"not found",0)</f>
+        <v>Application Developer</v>
+      </c>
+      <c r="O22" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P22" s="2" t="str">
+        <v>Mortgage</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>135000</v>
+      </c>
+      <c r="R22" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S22" s="2" t="str">
+        <v>Not Verified</v>
+      </c>
+      <c r="T22" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U22" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V22" s="2">
+        <v>35562</v>
+      </c>
+      <c r="W22" s="2">
+        <v>355619</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>64</v>
       </c>
@@ -3938,8 +4202,42 @@
       <c r="K23" s="2">
         <v>382595</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M23" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="N23" s="2" t="str" cm="1">
+        <f t="array" ref="N23:W23">_xlfn.XLOOKUP(M23,A7:A399,B7:K399,"not found",0)</f>
+        <v>None</v>
+      </c>
+      <c r="O23" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="P23" s="2" t="str">
+        <v>Mortgage</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>52800</v>
+      </c>
+      <c r="R23" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S23" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="T23" s="2" t="str">
+        <v>480xx</v>
+      </c>
+      <c r="U23" s="2" t="str">
+        <v>MI</v>
+      </c>
+      <c r="V23" s="2">
+        <v>21029</v>
+      </c>
+      <c r="W23" s="2">
+        <v>105146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>66</v>
       </c>
@@ -3973,8 +4271,42 @@
       <c r="K24" s="2">
         <v>28413</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="N24" s="2" t="str" cm="1">
+        <f t="array" ref="N24:W24">_xlfn.XLOOKUP(M24,A8:A400,B8:K400,"not found",0)</f>
+        <v>National Client Space Manager</v>
+      </c>
+      <c r="O24" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P24" s="2" t="str">
+        <v>Mortgage</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>86000</v>
+      </c>
+      <c r="R24" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S24" s="2" t="str">
+        <v>Source Verified</v>
+      </c>
+      <c r="T24" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U24" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V24" s="2">
+        <v>19868</v>
+      </c>
+      <c r="W24" s="2">
+        <v>298017</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>68</v>
       </c>
@@ -4008,8 +4340,42 @@
       <c r="K25" s="2">
         <v>40630</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M25" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="N25" s="2" t="str" cm="1">
+        <f t="array" ref="N25:W25">_xlfn.XLOOKUP(M25,A9:A401,B9:K401,"not found",0)</f>
+        <v xml:space="preserve">School Psychologist </v>
+      </c>
+      <c r="O25" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P25" s="2" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>90000</v>
+      </c>
+      <c r="R25" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S25" s="2" t="str">
+        <v>Verified</v>
+      </c>
+      <c r="T25" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U25" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V25" s="2">
+        <v>11132</v>
+      </c>
+      <c r="W25" s="2">
+        <v>144718</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>70</v>
       </c>
@@ -4043,8 +4409,42 @@
       <c r="K26" s="2">
         <v>111366</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="M26" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="N26" s="2" t="str" cm="1">
+        <f t="array" ref="N26:W26">_xlfn.XLOOKUP(M26,A10:A402,B10:K402,"not found",0)</f>
+        <v>Teacher</v>
+      </c>
+      <c r="O26" s="2" t="str">
+        <v>5 years</v>
+      </c>
+      <c r="P26" s="2" t="str">
+        <v>Mortgage</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>96000</v>
+      </c>
+      <c r="R26" s="2" t="str">
+        <v>none</v>
+      </c>
+      <c r="S26" s="2" t="str">
+        <v>Not Verified</v>
+      </c>
+      <c r="T26" s="2" t="str">
+        <v>109xx</v>
+      </c>
+      <c r="U26" s="2" t="str">
+        <v>NY</v>
+      </c>
+      <c r="V26" s="2">
+        <v>54834</v>
+      </c>
+      <c r="W26" s="2">
+        <v>383838</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>72</v>
       </c>
@@ -4079,7 +4479,7 @@
         <v>28747</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>74</v>
       </c>
@@ -4114,7 +4514,7 @@
         <v>20751</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>75</v>
       </c>
@@ -4149,7 +4549,7 @@
         <v>204961</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>77</v>
       </c>
@@ -4184,7 +4584,7 @@
         <v>40001</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>79</v>
       </c>
@@ -4219,7 +4619,7 @@
         <v>8562</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>81</v>
       </c>
@@ -16926,7 +17326,7 @@
     </row>
     <row r="395" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E395">
-        <f t="shared" ref="C395:I395" si="1">SUM(E1:E394)</f>
+        <f t="shared" ref="E395:F395" si="1">SUM(E1:E394)</f>
         <v>38335069.949000001</v>
       </c>
       <c r="F395">
@@ -16943,6 +17343,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
correct some mistake in excel
</commit_message>
<xml_diff>
--- a/finance_customer.csv.xlsx
+++ b/finance_customer.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pandas\Finance data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD10826B-74FE-45F1-985F-B20A4F0010F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413594EE-6A91-4D9F-89EB-E30AB5C43CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9802DE5F-B1D8-4319-BDEA-30F1B831059A}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3145" uniqueCount="730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3144" uniqueCount="730">
   <si>
     <t>customer_id</t>
   </si>
@@ -16495,16 +16495,15 @@
   <dimension ref="A1:V395"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" style="5" customWidth="1"/>
-    <col min="7" max="7" width="8" style="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" style="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.44140625" bestFit="1" customWidth="1"/>
@@ -17983,24 +17982,22 @@
       <c r="P33" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="Q33" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="R33" s="1" t="s">
+      <c r="Q33" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="R33" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="S33" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="T33" s="10" t="s">
         <v>8</v>
       </c>
+      <c r="T33" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="U33" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="V33" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="V33" s="1"/>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">

</xml_diff>